<commit_message>
bulk statusupload final integration
</commit_message>
<xml_diff>
--- a/Jobs/Tasks/FileProcess/StatusUpdateExcel.xlsx
+++ b/Jobs/Tasks/FileProcess/StatusUpdateExcel.xlsx
@@ -35,10 +35,10 @@
     <t>Status</t>
   </si>
   <si>
-    <t>AG033</t>
+    <t>Terminate</t>
   </si>
   <si>
-    <t>Terminate</t>
+    <t>AGT002</t>
   </si>
 </sst>
 </file>
@@ -387,13 +387,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" s="2">
-        <v>46070</v>
+        <v>46100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>